<commit_message>
new commit - simualtion
</commit_message>
<xml_diff>
--- a/balance_generate/dictionaries/client_type.xlsx
+++ b/balance_generate/dictionaries/client_type.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_generate\dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7B68F9-DD28-4E69-AB84-D7C0DA098911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13CA154-42C2-44D7-88C5-25DE3790B92A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6400" yWindow="1820" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>IND</t>
   </si>
@@ -73,36 +73,6 @@
   </si>
   <si>
     <t>client_type</t>
-  </si>
-  <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>05</t>
-  </si>
-  <si>
-    <t>06</t>
-  </si>
-  <si>
-    <t>07</t>
-  </si>
-  <si>
-    <t>08</t>
-  </si>
-  <si>
-    <t>09</t>
-  </si>
-  <si>
-    <t>10</t>
   </si>
 </sst>
 </file>
@@ -140,7 +110,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,80 +408,80 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
+      <c r="A2" s="1">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>17</v>
+      <c r="A3" s="1">
+        <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
+      <c r="A4" s="1">
+        <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>19</v>
+      <c r="A5" s="1">
+        <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>20</v>
+      <c r="A6" s="1">
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>21</v>
+      <c r="A7" s="1">
+        <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>22</v>
+      <c r="A8" s="1">
+        <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>23</v>
+      <c r="A9" s="1">
+        <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>24</v>
+      <c r="A10" s="1">
+        <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>25</v>
+      <c r="A11" s="1">
+        <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>10</v>

</xml_diff>